<commit_message>
fix(r5.2): explicit manager_required labels and field trial kit
</commit_message>
<xml_diff>
--- a/docs/R5-PILOT-EVENTS-TEMPLATE.xlsx
+++ b/docs/R5-PILOT-EVENTS-TEMPLATE.xlsx
@@ -83,6 +83,11 @@
       </c>
       <c r="O1" t="inlineStr">
         <is>
+          <t>manager_required</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
           <t>manager_sufficiency</t>
         </is>
       </c>
@@ -163,6 +168,11 @@
           <t/>
         </is>
       </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -240,6 +250,11 @@
           <t/>
         </is>
       </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -317,6 +332,11 @@
           <t/>
         </is>
       </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -390,6 +410,11 @@
         </is>
       </c>
       <c r="O5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
         <is>
           <t/>
         </is>

</xml_diff>

<commit_message>
fix(r5.2): manager_required provenance, frozen model and field start gate
</commit_message>
<xml_diff>
--- a/docs/R5-PILOT-EVENTS-TEMPLATE.xlsx
+++ b/docs/R5-PILOT-EVENTS-TEMPLATE.xlsx
@@ -88,6 +88,11 @@
       </c>
       <c r="P1" t="inlineStr">
         <is>
+          <t>manager_required_reason</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
           <t>manager_sufficiency</t>
         </is>
       </c>
@@ -173,6 +178,11 @@
           <t/>
         </is>
       </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -255,6 +265,11 @@
           <t/>
         </is>
       </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -337,6 +352,11 @@
           <t/>
         </is>
       </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -415,6 +435,11 @@
         </is>
       </c>
       <c r="P5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
         <is>
           <t/>
         </is>

</xml_diff>